<commit_message>
fix: forzar recalculo completo y verificar auxiliares y probabilidades XLSX
</commit_message>
<xml_diff>
--- a/soluciones/hojas/Ejercicio2.xlsx
+++ b/soluciones/hojas/Ejercicio2.xlsx
@@ -639,7 +639,7 @@
       </c>
       <c r="B9" s="0" t="n">
         <f aca="false">B6^2*B4</f>
-        <v>0</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -648,7 +648,7 @@
       </c>
       <c r="B10" s="0" t="n">
         <f aca="false">SQRT(B9)</f>
-        <v>0</v>
+        <v>0.014142135623731</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -657,7 +657,7 @@
       </c>
       <c r="B11" s="0" t="n">
         <f aca="false">IF(B10=0,0,(B2-B3)/B10)</f>
-        <v>0</v>
+        <v>-0.14142135623731</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -665,8 +665,8 @@
         <v>23</v>
       </c>
       <c r="B12" s="0" t="n">
-        <f aca="false">norm.s.dist(B11,TRUE())</f>
-        <v>0</v>
+        <f aca="false">NORMDIST(B11,0,1,TRUE())</f>
+        <v>0.443768541990857</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -674,8 +674,8 @@
         <v>24</v>
       </c>
       <c r="B13" s="0" t="n">
-        <f aca="false">norm.s.dist(B11,FALSE())</f>
-        <v>0</v>
+        <f aca="false">NORMDIST(B11,0,1,FALSE())</f>
+        <v>0.394972738386952</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -684,7 +684,7 @@
       </c>
       <c r="B14" s="0" t="n">
         <f aca="false">IF(B10=0,MAX(B2-B3,0),(B2-B3)*B12+B10*B13)</f>
-        <v>0</v>
+        <v>0.00469822094996297</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -693,7 +693,7 @@
       </c>
       <c r="B15" s="0" t="n">
         <f aca="false">IF(B10=0,MAX(B3-B2,0),(B3-B2)*(1-B12)+B10*B13)</f>
-        <v>0</v>
+        <v>0.00669822094996297</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -702,7 +702,7 @@
       </c>
       <c r="B16" s="0" t="n">
         <f aca="false">B7*(1+B5*B2)</f>
-        <v>0</v>
+        <v>0.941659638623481</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -747,7 +747,7 @@
       </c>
       <c r="B21" s="0" t="n">
         <f aca="false">B2+B5*B9/(1+B5*B2)</f>
-        <v>0</v>
+        <v>0.0300985221674877</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>